<commit_message>
a jednak jeszcze ostatnia popraweczka danych w excelach
</commit_message>
<xml_diff>
--- a/training_results_DENSENET_CIFAR_augumentacja.xlsx
+++ b/training_results_DENSENET_CIFAR_augumentacja.xlsx
@@ -490,62 +490,12 @@
         <v>cuda</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>Densenet121</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>SGD</v>
       </c>
       <c r="P2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2026-05-25 23:00:01</v>
-      </c>
-      <c r="B3" t="str">
-        <v>CIFAR10</v>
-      </c>
-      <c r="C3" t="str">
-        <v>64</v>
-      </c>
-      <c r="D3" t="str">
-        <v>20</v>
-      </c>
-      <c r="E3" t="str">
-        <v>20</v>
-      </c>
-      <c r="F3" t="str">
-        <v>0.01</v>
-      </c>
-      <c r="G3" t="str">
-        <v>5</v>
-      </c>
-      <c r="H3" t="str">
-        <v>98.93</v>
-      </c>
-      <c r="I3" t="str">
-        <v>97.64</v>
-      </c>
-      <c r="J3" t="str">
-        <v>92.91</v>
-      </c>
-      <c r="K3" t="str">
-        <v>0.5584</v>
-      </c>
-      <c r="L3" t="str">
-        <v>models/densenet_model_augumentacja_cifar10_64batch_20epochs_0.01lr.pth</v>
-      </c>
-      <c r="M3" t="str">
-        <v>cuda</v>
-      </c>
-      <c r="N3" t="str">
-        <v>ViT Small Patch16 224</v>
-      </c>
-      <c r="O3" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="P3" t="str">
         <v>CosineAnnealingLR</v>
       </c>
     </row>

</xml_diff>